<commit_message>
Update mapping to real YSELL API field structure
- title (not name), purchase_price (not suppliers), image (direct string)
- Fetch manufacturers via /api/v1/manufacturer to resolve manufacturer_id → name
- Viox check uses manufacturer name from API (manufacturer_id lookup)
- parseTitleForCompatibility(): extract brands/models from "wie BRAND NUM" pattern
  - brands: letter-only tokens after "wie" (handles IGNIS, EGO, Bauknecht)
  - models: digit-containing tokens, deduplicated, max 3
- Fallback: extract part numbers from title when no "wie" pattern present
- sample_products.json updated to mirror real API shape
- sample_manufacturers.json added for --sample test mode

https://claude.ai/code/session_013CC3uQiZgCtv7kaNkq2QqP
</commit_message>
<xml_diff>
--- a/flat_filled.xlsx
+++ b/flat_filled.xlsx
@@ -95,10 +95,10 @@
     <t>Add (SiteID=Germany|Country=DE|Currency=EUR|Version=941)</t>
   </si>
   <si>
-    <t>1001-MP</t>
-  </si>
-  <si>
-    <t>Umwälzpumpe für Geschirrspüler Bosch</t>
+    <t>2-MP</t>
+  </si>
+  <si>
+    <t>Aufbewahrungstasche für Zubehör Scheiben Bosch 00653180 von Küchmaschine</t>
   </si>
   <si>
     <t>Neu</t>
@@ -122,88 +122,88 @@
     <t>UK Gutschein</t>
   </si>
   <si>
-    <t>https://cdn.ysell.pro/products/1001/main.jpg</t>
+    <t>https://4457.test1.ysell.pro/product_images/2/Удалить.jpg</t>
   </si>
   <si>
     <t>Viox</t>
   </si>
   <si>
-    <t>Umwälzpumpe</t>
-  </si>
-  <si>
-    <t>Schwarz</t>
-  </si>
-  <si>
-    <t>Kunststoff</t>
-  </si>
-  <si>
-    <t>Bosch, Siemens, Neff</t>
-  </si>
-  <si>
-    <t>SMV50E90EU, SMV51E10EU, SMV53L00EU</t>
-  </si>
-  <si>
-    <t>VP-1001</t>
+    <t>Aufbewahrungstasche</t>
+  </si>
+  <si>
+    <t>00653180</t>
   </si>
   <si>
     <t>Vollintegriert</t>
   </si>
   <si>
-    <t>sku=DC31-00030A</t>
-  </si>
-  <si>
-    <t>Ablaufpumpe Waschmaschine Samsung</t>
-  </si>
-  <si>
-    <t>https://cdn.ysell.pro/products/1002/main.jpg</t>
-  </si>
-  <si>
-    <t>Samsung</t>
-  </si>
-  <si>
-    <t>Ablaufpumpe</t>
-  </si>
-  <si>
-    <t>Grau</t>
-  </si>
-  <si>
-    <t>ABS-Kunststoff</t>
-  </si>
-  <si>
-    <t>WF70F5E0W2W, WF80F5E4W4W, WF90F5E6QW4</t>
-  </si>
-  <si>
-    <t>DC31-00030A</t>
-  </si>
-  <si>
-    <t>1003-MP</t>
-  </si>
-  <si>
-    <t>Türdichtung Kühlschrank Whirlpool</t>
-  </si>
-  <si>
-    <t>Gebraucht</t>
-  </si>
-  <si>
-    <t>https://cdn.ysell.pro/products/1003/main.jpg</t>
-  </si>
-  <si>
-    <t>Türdichtung</t>
-  </si>
-  <si>
-    <t>Weiß</t>
-  </si>
-  <si>
-    <t>EPDM-Gummi</t>
-  </si>
-  <si>
-    <t>Whirlpool, Bauknecht</t>
-  </si>
-  <si>
-    <t>ARG590A, ARC4030, WBC3525A</t>
-  </si>
-  <si>
-    <t>VP-1003</t>
+    <t>p-4457-7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Seitenteil Halter Halterung rechts für Türfach Kühlschrank wie Liebherr 7433698 </t>
+  </si>
+  <si>
+    <t>https://4457.test1.ysell.pro/product_images/7/16342021668.jpeg</t>
+  </si>
+  <si>
+    <t>Original</t>
+  </si>
+  <si>
+    <t>Seitenteil</t>
+  </si>
+  <si>
+    <t>Liebherr</t>
+  </si>
+  <si>
+    <t>7433698, 9193354</t>
+  </si>
+  <si>
+    <t>p-4457-8</t>
+  </si>
+  <si>
+    <t>Spannrolle wie Bosch 00600436 für Zweibandmotor Trockner</t>
+  </si>
+  <si>
+    <t>https://4457.test1.ysell.pro/product_images/8/p-1-69678_1-1_info.jpg</t>
+  </si>
+  <si>
+    <t>Spannrolle</t>
+  </si>
+  <si>
+    <t>Bosch</t>
+  </si>
+  <si>
+    <t>00600436</t>
+  </si>
+  <si>
+    <t>p-4457-5</t>
+  </si>
+  <si>
+    <t>Heizung Oberhitze SoftGrill wie IGNIS 488000525918 EGO 20.40943.000 Bauknecht 48</t>
+  </si>
+  <si>
+    <t>https://4457.test1.ysell.pro/product_images/5/p-1-66796_1-2_info_DE.jpg</t>
+  </si>
+  <si>
+    <t>Heizung</t>
+  </si>
+  <si>
+    <t>IGNIS, EGO, Bauknecht</t>
+  </si>
+  <si>
+    <t>488000525918, 20.40943.000, 481225998522</t>
+  </si>
+  <si>
+    <t>12-MP</t>
+  </si>
+  <si>
+    <t>Bosch Siemens 17002715 / 17001433 Backblech Fettpfanne Grillpfanne 455x375x39(33</t>
+  </si>
+  <si>
+    <t>https://4457.test1.ysell.pro/product_images/12/13682.jpg</t>
+  </si>
+  <si>
+    <t>17002715, 17001433</t>
   </si>
 </sst>
 </file>
@@ -553,7 +553,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:Y4"/>
+  <dimension ref="A1:Y6"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="9.283" customWidth="true" style="0"/>
@@ -667,9 +667,6 @@
       <c r="B2" t="s">
         <v>26</v>
       </c>
-      <c r="C2">
-        <v>20715</v>
-      </c>
       <c r="D2" t="s">
         <v>27</v>
       </c>
@@ -679,9 +676,6 @@
       <c r="F2" t="s">
         <v>28</v>
       </c>
-      <c r="G2">
-        <v>12.5</v>
-      </c>
       <c r="H2">
         <v>1</v>
       </c>
@@ -718,23 +712,14 @@
       <c r="S2" t="s">
         <v>37</v>
       </c>
-      <c r="T2" t="s">
+      <c r="W2" t="s">
         <v>38</v>
       </c>
-      <c r="U2" t="s">
+      <c r="X2" t="s">
+        <v>38</v>
+      </c>
+      <c r="Y2" t="s">
         <v>39</v>
-      </c>
-      <c r="V2" t="s">
-        <v>40</v>
-      </c>
-      <c r="W2" t="s">
-        <v>41</v>
-      </c>
-      <c r="X2" t="s">
-        <v>42</v>
-      </c>
-      <c r="Y2" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="3" spans="1:25">
@@ -742,13 +727,10 @@
         <v>25</v>
       </c>
       <c r="B3" t="s">
-        <v>44</v>
-      </c>
-      <c r="C3">
-        <v>20715</v>
+        <v>40</v>
       </c>
       <c r="D3" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="E3">
         <v>1000</v>
@@ -757,7 +739,7 @@
         <v>28</v>
       </c>
       <c r="G3">
-        <v>18.9</v>
+        <v>3.74</v>
       </c>
       <c r="H3">
         <v>1</v>
@@ -781,37 +763,31 @@
         <v>34</v>
       </c>
       <c r="O3" t="s">
+        <v>42</v>
+      </c>
+      <c r="P3" t="s">
+        <v>43</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>43</v>
+      </c>
+      <c r="R3" t="s">
+        <v>44</v>
+      </c>
+      <c r="S3" t="s">
+        <v>44</v>
+      </c>
+      <c r="V3" t="s">
+        <v>45</v>
+      </c>
+      <c r="W3" t="s">
         <v>46</v>
       </c>
-      <c r="P3" t="s">
-        <v>47</v>
-      </c>
-      <c r="Q3" t="s">
-        <v>47</v>
-      </c>
-      <c r="R3" t="s">
-        <v>48</v>
-      </c>
-      <c r="S3" t="s">
-        <v>48</v>
-      </c>
-      <c r="T3" t="s">
-        <v>49</v>
-      </c>
-      <c r="U3" t="s">
-        <v>50</v>
-      </c>
-      <c r="V3" t="s">
-        <v>47</v>
-      </c>
-      <c r="W3" t="s">
-        <v>51</v>
-      </c>
-      <c r="X3" t="s">
-        <v>52</v>
+      <c r="X3">
+        <v>7433698</v>
       </c>
       <c r="Y3" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
     </row>
     <row r="4" spans="1:25">
@@ -819,22 +795,19 @@
         <v>25</v>
       </c>
       <c r="B4" t="s">
-        <v>53</v>
-      </c>
-      <c r="C4">
-        <v>43576</v>
+        <v>47</v>
       </c>
       <c r="D4" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="E4">
-        <v>3000</v>
+        <v>1000</v>
       </c>
       <c r="F4" t="s">
-        <v>55</v>
+        <v>28</v>
       </c>
       <c r="G4">
-        <v>9.99</v>
+        <v>3.96</v>
       </c>
       <c r="H4">
         <v>1</v>
@@ -858,37 +831,161 @@
         <v>34</v>
       </c>
       <c r="O4" t="s">
+        <v>49</v>
+      </c>
+      <c r="P4" t="s">
+        <v>43</v>
+      </c>
+      <c r="Q4" t="s">
+        <v>43</v>
+      </c>
+      <c r="R4" t="s">
+        <v>50</v>
+      </c>
+      <c r="S4" t="s">
+        <v>50</v>
+      </c>
+      <c r="V4" t="s">
+        <v>51</v>
+      </c>
+      <c r="W4" t="s">
+        <v>52</v>
+      </c>
+      <c r="X4" t="s">
+        <v>52</v>
+      </c>
+      <c r="Y4" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="5" spans="1:25">
+      <c r="A5" t="s">
+        <v>25</v>
+      </c>
+      <c r="B5" t="s">
+        <v>53</v>
+      </c>
+      <c r="D5" t="s">
+        <v>54</v>
+      </c>
+      <c r="E5">
+        <v>1000</v>
+      </c>
+      <c r="F5" t="s">
+        <v>28</v>
+      </c>
+      <c r="H5">
+        <v>1</v>
+      </c>
+      <c r="I5" t="s">
+        <v>29</v>
+      </c>
+      <c r="J5" t="s">
+        <v>30</v>
+      </c>
+      <c r="K5" t="s">
+        <v>31</v>
+      </c>
+      <c r="L5" t="s">
+        <v>32</v>
+      </c>
+      <c r="M5" t="s">
+        <v>33</v>
+      </c>
+      <c r="N5" t="s">
+        <v>34</v>
+      </c>
+      <c r="O5" t="s">
+        <v>55</v>
+      </c>
+      <c r="P5" t="s">
+        <v>43</v>
+      </c>
+      <c r="Q5" t="s">
+        <v>43</v>
+      </c>
+      <c r="R5" t="s">
         <v>56</v>
       </c>
-      <c r="P4" t="s">
+      <c r="S5" t="s">
+        <v>56</v>
+      </c>
+      <c r="V5" t="s">
+        <v>57</v>
+      </c>
+      <c r="W5" t="s">
+        <v>58</v>
+      </c>
+      <c r="X5">
+        <v>488000525918</v>
+      </c>
+      <c r="Y5" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="6" spans="1:25">
+      <c r="A6" t="s">
+        <v>25</v>
+      </c>
+      <c r="B6" t="s">
+        <v>59</v>
+      </c>
+      <c r="D6" t="s">
+        <v>60</v>
+      </c>
+      <c r="E6">
+        <v>1000</v>
+      </c>
+      <c r="F6" t="s">
+        <v>28</v>
+      </c>
+      <c r="G6">
+        <v>18.19</v>
+      </c>
+      <c r="H6">
+        <v>1</v>
+      </c>
+      <c r="I6" t="s">
+        <v>29</v>
+      </c>
+      <c r="J6" t="s">
+        <v>30</v>
+      </c>
+      <c r="K6" t="s">
+        <v>31</v>
+      </c>
+      <c r="L6" t="s">
+        <v>32</v>
+      </c>
+      <c r="M6" t="s">
+        <v>33</v>
+      </c>
+      <c r="N6" t="s">
+        <v>34</v>
+      </c>
+      <c r="O6" t="s">
+        <v>61</v>
+      </c>
+      <c r="P6" t="s">
         <v>36</v>
       </c>
-      <c r="Q4" t="s">
+      <c r="Q6" t="s">
         <v>36</v>
       </c>
-      <c r="R4" t="s">
-        <v>57</v>
-      </c>
-      <c r="S4" t="s">
-        <v>57</v>
-      </c>
-      <c r="T4" t="s">
-        <v>58</v>
-      </c>
-      <c r="U4" t="s">
-        <v>59</v>
-      </c>
-      <c r="V4" t="s">
-        <v>60</v>
-      </c>
-      <c r="W4" t="s">
-        <v>61</v>
-      </c>
-      <c r="X4" t="s">
+      <c r="R6" t="s">
+        <v>51</v>
+      </c>
+      <c r="S6" t="s">
+        <v>51</v>
+      </c>
+      <c r="W6" t="s">
         <v>62</v>
       </c>
-      <c r="Y4" t="s">
-        <v>43</v>
+      <c r="X6">
+        <v>17002715</v>
+      </c>
+      <c r="Y6" t="s">
+        <v>39</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add category lookup (A+B) and HTML description generation
Category:
- Variant A: keyword map covering 7 appliance categories
  (Geschirrspüler→116026, Waschmaschine/Trockner→99697,
   Kühlschrank→184666, Backofen/Herd→43566, Dunstabzug→71253,
   Kaffeemaschine/Staubsauger/Fleischwolf→99565)
- Variant B: eBay.de scraping fallback (_sacat regex from search page)
- Combined: A first, B only on keyword miss; eBay results cached

Description:
- Full HTML template matching Html.html structure from repo
- Dynamic: product title, image, OEM numbers, brand compatibility
- Static: header/footer/CSS from ersatzteil-check.de template
- Added Description column D; all other columns shifted D→E…Y→Z

Also:
- Fixed getCategoryByKeywords() return type (int keys cast to string)
- Added küchmaschine/zahnrad to keyword map
- Updated verify_output.php for new column layout
- getHighestDataRow() used in verify to avoid empty column scan

https://claude.ai/code/session_013CC3uQiZgCtv7kaNkq2QqP
</commit_message>
<xml_diff>
--- a/flat_filled.xlsx
+++ b/flat_filled.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="69">
   <si>
     <t>*Action</t>
   </si>
@@ -26,6 +26,9 @@
     <t>*Category</t>
   </si>
   <si>
+    <t>Description</t>
+  </si>
+  <si>
     <t>*Title</t>
   </si>
   <si>
@@ -98,6 +101,144 @@
     <t>2-MP</t>
   </si>
   <si>
+    <t>&lt;!DOCTYPE html&gt;
+&lt;html&gt;
+&lt;head&gt;
+    &lt;meta charset="utf-8"&gt;
+    &lt;meta name="viewport" content="width=device-width, initial-scale=1"&gt;
+    &lt;title&gt;eBay&lt;/title&gt;
+    &lt;link rel="preconnect" href="https://fonts.googleapis.com"&gt;
+    &lt;link rel="preconnect" href="https://fonts.gstatic.com" crossorigin&gt;
+    &lt;link href="https://fonts.googleapis.com/css2?family=Inter:wght@400;600&amp;display=swap" rel="stylesheet"&gt;
+    &lt;link rel="stylesheet" href="https://ersatzteil-check.de/ebay_template/css/style.css"&gt;
+    &lt;link rel="stylesheet" href="https://ersatzteil-check.de/ebay_template/css/new_style.css"&gt;
+    &lt;link href="https://cdn.jsdelivr.net/npm/bootstrap@5.3.2/dist/css/bootstrap.min.css" rel="stylesheet" crossorigin="anonymous"&gt;
+&lt;/head&gt;
+&lt;body&gt;
+&lt;div class="ebay-content"&gt;
+    &lt;header class="container header"&gt;
+        &lt;img src="https://ersatzteil-check.de/ebay_template/img/logo.svg"&gt;
+        &lt;div class="menu"&gt;
+            &lt;a class="menu-item" href="https://www.ebay.de/str/bremenhaushalt"&gt;Über uns&lt;/a&gt;
+            &lt;a class="menu-item" href="https://www.ebay.de/cnt/intermediatedFAQ?requested=ersatzteil-check-de"&gt;Kontakt&lt;/a&gt;
+            &lt;a class="menu-item" href="https://www.ebay.de/str/bremenhaushalt?_tab=2"&gt;Bewertungen&lt;/a&gt;
+            &lt;a class="menu-item-btn" href="https://www.ebay.de/str/bremenhaushalt"&gt;eBay Shop&lt;/a&gt;
+        &lt;/div&gt;
+    &lt;/header&gt;
+    &lt;div class="container"&gt;
+        &lt;img class="banner" src="https://ersatzteil-check.de/ebay_template/img/banner.png"&gt;
+    &lt;/div&gt;
+    &lt;div class="container gears"&gt;
+        &lt;div class="column-3"&gt;
+            &lt;img src="https://ersatzteil-check.de/ebay_template/img/Group1.png"&gt;
+            &lt;p&gt;Schnelle Lieferung&lt;/p&gt;
+        &lt;/div&gt;
+        &lt;div class="column-3"&gt;
+            &lt;img src="https://ersatzteil-check.de/ebay_template/img/Group2.png"&gt;
+            &lt;p&gt;Riesige Auswahl&lt;/p&gt;
+        &lt;/div&gt;
+        &lt;div class="column-3"&gt;
+            &lt;img src="https://ersatzteil-check.de/ebay_template/img/Group3.png"&gt;
+            &lt;p&gt;30 Tage Widerruffrist&lt;/p&gt;
+        &lt;/div&gt;
+    &lt;/div&gt;
+    &lt;footer class="footer"&gt;
+        &lt;div class="container"&gt;
+            &lt;div class="footer-menu"&gt;
+                &lt;a class="footer-item" href="https://www.ebay.de/sch/i.html?_ssn=ersatzteil-check-de&amp;store_name=bremenhaushalt&amp;_oac=1&amp;_trksid=p4429486.m3561.l2562"&gt;Alle Artikel&lt;/a&gt;
+                &lt;a class="footer-item" href="https://www.ebay.de/str/bremenhaushalt/Backofen-Herdteile/_i.html?_sacat=43566"&gt;Backofen- &amp;amp; Herdeteile&lt;/a&gt;
+                &lt;a class="footer-item" href="https://www.ebay.de/str/bremenhaushalt/Waschmaschinen-Trocknerteile/_i.html?_sacat=99697"&gt;Waschmaschinen- &amp;amp; Trocknerteile&lt;/a&gt;
+                &lt;a class="footer-item" href="https://www.ebay.de/str/bremenhaushalt/Gefriergerate-Kuhlschrankteile/_i.html?_sacat=184666"&gt;Gefriergeräte- &amp;amp; Kühlschrankteile&lt;/a&gt;
+                &lt;a class="footer-item" href="https://www.ebay.de/str/bremenhaushalt/Geschirrspulerteile/_i.html?_sacat=116026"&gt;Geschirrspülerteile&lt;/a&gt;
+                &lt;a class="footer-item" href="https://www.ebay.de/str/bremenhaushalt/Ersatzteile/_i.html?_sacat=99565"&gt;Kaffeemaschinen Ersatzteile&lt;/a&gt;
+                &lt;a class="footer-item" href="https://www.ebay.de/str/bremenhaushalt/Dunstabzugshauben/_i.html?_sacat=71253"&gt;Dunstabzugshauben Ersatzteile&lt;/a&gt;
+            &lt;/div&gt;
+        &lt;/div&gt;
+    &lt;/footer&gt;
+&lt;/div&gt;
+&lt;div class="container-fluid content-bg" align="center"&gt;
+    &lt;br/&gt;
+    &lt;div class="container"&gt;
+        &lt;div class="row"&gt;
+            &lt;div class="col-md-12 maincontent"&gt;
+                &lt;div class="row top_head"&gt;
+                    &lt;h1&gt;&lt;b style="color:#ff0000"&gt;Aufbewahrungstasche für Zubehör Scheiben Bosch 00653180 von Küchmaschine&lt;/b&gt;&lt;/h1&gt;
+                &lt;/div&gt;
+                &lt;div class="textbox main"&gt;
+                    &lt;div class="row artdesc"&gt;
+                        &lt;div class="col-md-6 artdesc-2"&gt;
+                            &lt;div class="image-gallery"&gt;
+                                &lt;div class="big-image"&gt;
+                                    &lt;img id="default" src="https://4457.test1.ysell.pro/product_images/2/Удалить.jpg"/&gt;
+                                &lt;/div&gt;
+                            &lt;/div&gt;
+                        &lt;/div&gt;
+                        &lt;div class="col-md-6 artdesc-3"&gt;
+                            &lt;div class="right_info"&gt;
+                                &lt;div class="row"&gt;
+                                    &lt;div class="col"&gt;
+                                        &lt;a href="#" class="button-1" id="ersatz-tocart"&gt;
+                                            &lt;img src="https://ersatzteil-check.de/ebay_template/img/cart.svg" alt=""&gt;
+                                            Kaufen
+                                        &lt;/a&gt;
+                                    &lt;/div&gt;
+                                    &lt;div class="col"&gt;
+                                        &lt;a href="#" class="button-2" id="ersatz-towatch"&gt;
+                                            &lt;img src="https://ersatzteil-check.de/ebay_template/img/globalization.svg" alt=""&gt;
+                                            Beobachten
+                                        &lt;/a&gt;
+                                    &lt;/div&gt;
+                                    &lt;div class="col"&gt;
+                                        &lt;a href="#" class="button-3" id="ersatz-toask"&gt;
+                                            &lt;img src="https://ersatzteil-check.de/ebay_template/img/support.svg" alt=""&gt;
+                                            Frage stellen
+                                        &lt;/a&gt;
+                                    &lt;/div&gt;
+                                &lt;/div&gt;
+                                &lt;ul style="list-style-type:none; padding-left:0;"&gt;
+                                    &lt;li style="color:#ff0000;font-weight:700"&gt;&amp;#9989; &lt;b&gt;Originalgetreue Passform:&lt;/b&gt; Passend als Ersatz für Artikel-Nr.: 00653180&lt;/li&gt;
+                                    &lt;li style="color:#ff0000;font-weight:700"&gt;&amp;#9989; &lt;b&gt;Vielseitig einsetzbar:&lt;/b&gt; Geeignet als Ersatzteil für viele gängige Haushaltsgeräte&lt;/li&gt;
+                                    &lt;li style="color:#ff0000;font-weight:700"&gt;&amp;#9989; &lt;b&gt;Geprüfte Qualität:&lt;/b&gt; Hochwertige Verarbeitung in vergleichbarer Hersteller-Qualität&lt;/li&gt;
+                                    &lt;li style="color:#ff0000;font-weight:700"&gt;&amp;#9989; &lt;b&gt;Schnelle Lösung:&lt;/b&gt; Direkter Austausch ohne Modifikation möglich&lt;/li&gt;
+                                    &lt;li style="color:#ff0000;font-weight:700"&gt;&amp;#9989; &lt;b&gt;Sind Sie unsicher?&lt;/b&gt; Wir helfen Ihnen gerne, das exakt benötigte Ersatzteil zu finden.&lt;/li&gt;
+                                &lt;/ul&gt;
+                            &lt;/div&gt;
+                        &lt;/div&gt;
+                    &lt;/div&gt;
+                &lt;/div&gt;
+                &lt;div class="row bottom_text"&gt;
+                    &lt;div class="col-md-12"&gt;
+                        &lt;div class="tbc-1"&gt;
+                            &lt;h2&gt;Beschreibung&lt;/h2&gt;
+                            &lt;b style="color:#ff0000"&gt;Aufbewahrungstasche für Zubehör Scheiben Bosch 00653180 von Küchmaschine&lt;/b&gt;&lt;br/&gt;&lt;br/&gt;
+                            &lt;span style="color:#ff0000"&gt;Dieser Artikel ist ein hochwertiges Ersatzteil für Haushaltsgeräte. Er entspricht den Original-Spezifikationen und eignet sich als direkter Austausch.&lt;/span&gt;&lt;br/&gt;&lt;br/&gt;
+                            Wir sind ein professioneller Hersteller und Vertreiber von Original-Ersatzteilen und Alternativprodukten für Haushaltsgeräte. Egal ob Waschmaschine, Herd oder Kühlschrank: Wir haben diverse preisgünstige Original- und Alternativteile in vergleichbarer Hersteller-Qualität im Angebot. Überzeugen Sie sich selbst von der Wertigkeit unserer Ersatzteile und verschaffen Sie Ihrem Haushaltsgerät ein zweites Leben.&lt;br/&gt;&lt;br/&gt;
+                            &lt;b&gt;Kompatibel mit:&lt;/b&gt;&lt;br/&gt;
+                            &lt;span style="color:#ff0000"&gt;00653180&lt;/span&gt;
+                        &lt;/div&gt;
+                    &lt;/div&gt;
+                &lt;/div&gt;
+                &lt;div class="row bottom_text"&gt;
+                    &lt;div class="col-md-12"&gt;
+                        &lt;div class="tbc-2"&gt;
+                            &lt;h2&gt;Zahlungsoptionen&lt;/h2&gt;
+                            &lt;img src="https://ersatzteil-check.de/ebay_template/img/zahlung-paypal_n.png"&gt;
+                            &lt;img src="https://ersatzteil-check.de/ebay_template/img/zahlung-ueberweisung_n.png"&gt;
+                        &lt;/div&gt;
+                        &lt;div class="tbc-3"&gt;
+                            &lt;h2&gt;Versandoptionen&lt;/h2&gt;
+                            &lt;img src="https://ersatzteil-check.de/ebay_template/img/versand-dhl_n.png"&gt;
+                        &lt;/div&gt;
+                    &lt;/div&gt;
+                &lt;/div&gt;
+            &lt;/div&gt;
+        &lt;/div&gt;
+    &lt;/div&gt;
+&lt;/div&gt;
+&lt;/body&gt;
+&lt;/html&gt;</t>
+  </si>
+  <si>
     <t>Aufbewahrungstasche für Zubehör Scheiben Bosch 00653180 von Küchmaschine</t>
   </si>
   <si>
@@ -140,6 +281,144 @@
     <t>p-4457-7</t>
   </si>
   <si>
+    <t>&lt;!DOCTYPE html&gt;
+&lt;html&gt;
+&lt;head&gt;
+    &lt;meta charset="utf-8"&gt;
+    &lt;meta name="viewport" content="width=device-width, initial-scale=1"&gt;
+    &lt;title&gt;eBay&lt;/title&gt;
+    &lt;link rel="preconnect" href="https://fonts.googleapis.com"&gt;
+    &lt;link rel="preconnect" href="https://fonts.gstatic.com" crossorigin&gt;
+    &lt;link href="https://fonts.googleapis.com/css2?family=Inter:wght@400;600&amp;display=swap" rel="stylesheet"&gt;
+    &lt;link rel="stylesheet" href="https://ersatzteil-check.de/ebay_template/css/style.css"&gt;
+    &lt;link rel="stylesheet" href="https://ersatzteil-check.de/ebay_template/css/new_style.css"&gt;
+    &lt;link href="https://cdn.jsdelivr.net/npm/bootstrap@5.3.2/dist/css/bootstrap.min.css" rel="stylesheet" crossorigin="anonymous"&gt;
+&lt;/head&gt;
+&lt;body&gt;
+&lt;div class="ebay-content"&gt;
+    &lt;header class="container header"&gt;
+        &lt;img src="https://ersatzteil-check.de/ebay_template/img/logo.svg"&gt;
+        &lt;div class="menu"&gt;
+            &lt;a class="menu-item" href="https://www.ebay.de/str/bremenhaushalt"&gt;Über uns&lt;/a&gt;
+            &lt;a class="menu-item" href="https://www.ebay.de/cnt/intermediatedFAQ?requested=ersatzteil-check-de"&gt;Kontakt&lt;/a&gt;
+            &lt;a class="menu-item" href="https://www.ebay.de/str/bremenhaushalt?_tab=2"&gt;Bewertungen&lt;/a&gt;
+            &lt;a class="menu-item-btn" href="https://www.ebay.de/str/bremenhaushalt"&gt;eBay Shop&lt;/a&gt;
+        &lt;/div&gt;
+    &lt;/header&gt;
+    &lt;div class="container"&gt;
+        &lt;img class="banner" src="https://ersatzteil-check.de/ebay_template/img/banner.png"&gt;
+    &lt;/div&gt;
+    &lt;div class="container gears"&gt;
+        &lt;div class="column-3"&gt;
+            &lt;img src="https://ersatzteil-check.de/ebay_template/img/Group1.png"&gt;
+            &lt;p&gt;Schnelle Lieferung&lt;/p&gt;
+        &lt;/div&gt;
+        &lt;div class="column-3"&gt;
+            &lt;img src="https://ersatzteil-check.de/ebay_template/img/Group2.png"&gt;
+            &lt;p&gt;Riesige Auswahl&lt;/p&gt;
+        &lt;/div&gt;
+        &lt;div class="column-3"&gt;
+            &lt;img src="https://ersatzteil-check.de/ebay_template/img/Group3.png"&gt;
+            &lt;p&gt;30 Tage Widerruffrist&lt;/p&gt;
+        &lt;/div&gt;
+    &lt;/div&gt;
+    &lt;footer class="footer"&gt;
+        &lt;div class="container"&gt;
+            &lt;div class="footer-menu"&gt;
+                &lt;a class="footer-item" href="https://www.ebay.de/sch/i.html?_ssn=ersatzteil-check-de&amp;store_name=bremenhaushalt&amp;_oac=1&amp;_trksid=p4429486.m3561.l2562"&gt;Alle Artikel&lt;/a&gt;
+                &lt;a class="footer-item" href="https://www.ebay.de/str/bremenhaushalt/Backofen-Herdteile/_i.html?_sacat=43566"&gt;Backofen- &amp;amp; Herdeteile&lt;/a&gt;
+                &lt;a class="footer-item" href="https://www.ebay.de/str/bremenhaushalt/Waschmaschinen-Trocknerteile/_i.html?_sacat=99697"&gt;Waschmaschinen- &amp;amp; Trocknerteile&lt;/a&gt;
+                &lt;a class="footer-item" href="https://www.ebay.de/str/bremenhaushalt/Gefriergerate-Kuhlschrankteile/_i.html?_sacat=184666"&gt;Gefriergeräte- &amp;amp; Kühlschrankteile&lt;/a&gt;
+                &lt;a class="footer-item" href="https://www.ebay.de/str/bremenhaushalt/Geschirrspulerteile/_i.html?_sacat=116026"&gt;Geschirrspülerteile&lt;/a&gt;
+                &lt;a class="footer-item" href="https://www.ebay.de/str/bremenhaushalt/Ersatzteile/_i.html?_sacat=99565"&gt;Kaffeemaschinen Ersatzteile&lt;/a&gt;
+                &lt;a class="footer-item" href="https://www.ebay.de/str/bremenhaushalt/Dunstabzugshauben/_i.html?_sacat=71253"&gt;Dunstabzugshauben Ersatzteile&lt;/a&gt;
+            &lt;/div&gt;
+        &lt;/div&gt;
+    &lt;/footer&gt;
+&lt;/div&gt;
+&lt;div class="container-fluid content-bg" align="center"&gt;
+    &lt;br/&gt;
+    &lt;div class="container"&gt;
+        &lt;div class="row"&gt;
+            &lt;div class="col-md-12 maincontent"&gt;
+                &lt;div class="row top_head"&gt;
+                    &lt;h1&gt;&lt;b style="color:#ff0000"&gt;Seitenteil Halter Halterung rechts für Türfach Kühlschrank wie Liebherr 7433698 9193354&lt;/b&gt;&lt;/h1&gt;
+                &lt;/div&gt;
+                &lt;div class="textbox main"&gt;
+                    &lt;div class="row artdesc"&gt;
+                        &lt;div class="col-md-6 artdesc-2"&gt;
+                            &lt;div class="image-gallery"&gt;
+                                &lt;div class="big-image"&gt;
+                                    &lt;img id="default" src="https://4457.test1.ysell.pro/product_images/7/16342021668.jpeg"/&gt;
+                                &lt;/div&gt;
+                            &lt;/div&gt;
+                        &lt;/div&gt;
+                        &lt;div class="col-md-6 artdesc-3"&gt;
+                            &lt;div class="right_info"&gt;
+                                &lt;div class="row"&gt;
+                                    &lt;div class="col"&gt;
+                                        &lt;a href="#" class="button-1" id="ersatz-tocart"&gt;
+                                            &lt;img src="https://ersatzteil-check.de/ebay_template/img/cart.svg" alt=""&gt;
+                                            Kaufen
+                                        &lt;/a&gt;
+                                    &lt;/div&gt;
+                                    &lt;div class="col"&gt;
+                                        &lt;a href="#" class="button-2" id="ersatz-towatch"&gt;
+                                            &lt;img src="https://ersatzteil-check.de/ebay_template/img/globalization.svg" alt=""&gt;
+                                            Beobachten
+                                        &lt;/a&gt;
+                                    &lt;/div&gt;
+                                    &lt;div class="col"&gt;
+                                        &lt;a href="#" class="button-3" id="ersatz-toask"&gt;
+                                            &lt;img src="https://ersatzteil-check.de/ebay_template/img/support.svg" alt=""&gt;
+                                            Frage stellen
+                                        &lt;/a&gt;
+                                    &lt;/div&gt;
+                                &lt;/div&gt;
+                                &lt;ul style="list-style-type:none; padding-left:0;"&gt;
+                                    &lt;li style="color:#ff0000;font-weight:700"&gt;&amp;#9989; &lt;b&gt;Originalgetreue Passform:&lt;/b&gt; Passend als Ersatz für Artikel-Nr.: 7433698, 9193354&lt;/li&gt;
+                                    &lt;li style="color:#ff0000;font-weight:700"&gt;&amp;#9989; &lt;b&gt;Vielseitig einsetzbar:&lt;/b&gt; Kompatibel mit Produkten der Marke(n): Liebherr&lt;/li&gt;
+                                    &lt;li style="color:#ff0000;font-weight:700"&gt;&amp;#9989; &lt;b&gt;Geprüfte Qualität:&lt;/b&gt; Hochwertige Verarbeitung in vergleichbarer Hersteller-Qualität&lt;/li&gt;
+                                    &lt;li style="color:#ff0000;font-weight:700"&gt;&amp;#9989; &lt;b&gt;Schnelle Lösung:&lt;/b&gt; Direkter Austausch ohne Modifikation möglich&lt;/li&gt;
+                                    &lt;li style="color:#ff0000;font-weight:700"&gt;&amp;#9989; &lt;b&gt;Sind Sie unsicher?&lt;/b&gt; Wir helfen Ihnen gerne, das exakt benötigte Ersatzteil zu finden.&lt;/li&gt;
+                                &lt;/ul&gt;
+                            &lt;/div&gt;
+                        &lt;/div&gt;
+                    &lt;/div&gt;
+                &lt;/div&gt;
+                &lt;div class="row bottom_text"&gt;
+                    &lt;div class="col-md-12"&gt;
+                        &lt;div class="tbc-1"&gt;
+                            &lt;h2&gt;Beschreibung&lt;/h2&gt;
+                            &lt;b style="color:#ff0000"&gt;Seitenteil Halter Halterung rechts für Türfach Kühlschrank wie Liebherr 7433698 9193354&lt;/b&gt;&lt;br/&gt;&lt;br/&gt;
+                            &lt;span style="color:#ff0000"&gt;Dieser Artikel ist ein hochwertiges Ersatzteil, das kompatibel mit Geräten der Marke(n) Liebherr ist. Er entspricht den Original-Spezifikationen und eignet sich als direkter Austausch.&lt;/span&gt;&lt;br/&gt;&lt;br/&gt;
+                            Wir sind ein professioneller Hersteller und Vertreiber von Original-Ersatzteilen und Alternativprodukten für Haushaltsgeräte. Egal ob Waschmaschine, Herd oder Kühlschrank: Wir haben diverse preisgünstige Original- und Alternativteile in vergleichbarer Hersteller-Qualität im Angebot. Überzeugen Sie sich selbst von der Wertigkeit unserer Ersatzteile und verschaffen Sie Ihrem Haushaltsgerät ein zweites Leben.&lt;br/&gt;&lt;br/&gt;
+                            &lt;b&gt;Kompatibel mit:&lt;/b&gt;&lt;br/&gt;
+                            &lt;span style="color:#ff0000"&gt;7433698&lt;br/&gt;9193354&lt;/span&gt;
+                        &lt;/div&gt;
+                    &lt;/div&gt;
+                &lt;/div&gt;
+                &lt;div class="row bottom_text"&gt;
+                    &lt;div class="col-md-12"&gt;
+                        &lt;div class="tbc-2"&gt;
+                            &lt;h2&gt;Zahlungsoptionen&lt;/h2&gt;
+                            &lt;img src="https://ersatzteil-check.de/ebay_template/img/zahlung-paypal_n.png"&gt;
+                            &lt;img src="https://ersatzteil-check.de/ebay_template/img/zahlung-ueberweisung_n.png"&gt;
+                        &lt;/div&gt;
+                        &lt;div class="tbc-3"&gt;
+                            &lt;h2&gt;Versandoptionen&lt;/h2&gt;
+                            &lt;img src="https://ersatzteil-check.de/ebay_template/img/versand-dhl_n.png"&gt;
+                        &lt;/div&gt;
+                    &lt;/div&gt;
+                &lt;/div&gt;
+            &lt;/div&gt;
+        &lt;/div&gt;
+    &lt;/div&gt;
+&lt;/div&gt;
+&lt;/body&gt;
+&lt;/html&gt;</t>
+  </si>
+  <si>
     <t xml:space="preserve">Seitenteil Halter Halterung rechts für Türfach Kühlschrank wie Liebherr 7433698 </t>
   </si>
   <si>
@@ -161,6 +440,144 @@
     <t>p-4457-8</t>
   </si>
   <si>
+    <t>&lt;!DOCTYPE html&gt;
+&lt;html&gt;
+&lt;head&gt;
+    &lt;meta charset="utf-8"&gt;
+    &lt;meta name="viewport" content="width=device-width, initial-scale=1"&gt;
+    &lt;title&gt;eBay&lt;/title&gt;
+    &lt;link rel="preconnect" href="https://fonts.googleapis.com"&gt;
+    &lt;link rel="preconnect" href="https://fonts.gstatic.com" crossorigin&gt;
+    &lt;link href="https://fonts.googleapis.com/css2?family=Inter:wght@400;600&amp;display=swap" rel="stylesheet"&gt;
+    &lt;link rel="stylesheet" href="https://ersatzteil-check.de/ebay_template/css/style.css"&gt;
+    &lt;link rel="stylesheet" href="https://ersatzteil-check.de/ebay_template/css/new_style.css"&gt;
+    &lt;link href="https://cdn.jsdelivr.net/npm/bootstrap@5.3.2/dist/css/bootstrap.min.css" rel="stylesheet" crossorigin="anonymous"&gt;
+&lt;/head&gt;
+&lt;body&gt;
+&lt;div class="ebay-content"&gt;
+    &lt;header class="container header"&gt;
+        &lt;img src="https://ersatzteil-check.de/ebay_template/img/logo.svg"&gt;
+        &lt;div class="menu"&gt;
+            &lt;a class="menu-item" href="https://www.ebay.de/str/bremenhaushalt"&gt;Über uns&lt;/a&gt;
+            &lt;a class="menu-item" href="https://www.ebay.de/cnt/intermediatedFAQ?requested=ersatzteil-check-de"&gt;Kontakt&lt;/a&gt;
+            &lt;a class="menu-item" href="https://www.ebay.de/str/bremenhaushalt?_tab=2"&gt;Bewertungen&lt;/a&gt;
+            &lt;a class="menu-item-btn" href="https://www.ebay.de/str/bremenhaushalt"&gt;eBay Shop&lt;/a&gt;
+        &lt;/div&gt;
+    &lt;/header&gt;
+    &lt;div class="container"&gt;
+        &lt;img class="banner" src="https://ersatzteil-check.de/ebay_template/img/banner.png"&gt;
+    &lt;/div&gt;
+    &lt;div class="container gears"&gt;
+        &lt;div class="column-3"&gt;
+            &lt;img src="https://ersatzteil-check.de/ebay_template/img/Group1.png"&gt;
+            &lt;p&gt;Schnelle Lieferung&lt;/p&gt;
+        &lt;/div&gt;
+        &lt;div class="column-3"&gt;
+            &lt;img src="https://ersatzteil-check.de/ebay_template/img/Group2.png"&gt;
+            &lt;p&gt;Riesige Auswahl&lt;/p&gt;
+        &lt;/div&gt;
+        &lt;div class="column-3"&gt;
+            &lt;img src="https://ersatzteil-check.de/ebay_template/img/Group3.png"&gt;
+            &lt;p&gt;30 Tage Widerruffrist&lt;/p&gt;
+        &lt;/div&gt;
+    &lt;/div&gt;
+    &lt;footer class="footer"&gt;
+        &lt;div class="container"&gt;
+            &lt;div class="footer-menu"&gt;
+                &lt;a class="footer-item" href="https://www.ebay.de/sch/i.html?_ssn=ersatzteil-check-de&amp;store_name=bremenhaushalt&amp;_oac=1&amp;_trksid=p4429486.m3561.l2562"&gt;Alle Artikel&lt;/a&gt;
+                &lt;a class="footer-item" href="https://www.ebay.de/str/bremenhaushalt/Backofen-Herdteile/_i.html?_sacat=43566"&gt;Backofen- &amp;amp; Herdeteile&lt;/a&gt;
+                &lt;a class="footer-item" href="https://www.ebay.de/str/bremenhaushalt/Waschmaschinen-Trocknerteile/_i.html?_sacat=99697"&gt;Waschmaschinen- &amp;amp; Trocknerteile&lt;/a&gt;
+                &lt;a class="footer-item" href="https://www.ebay.de/str/bremenhaushalt/Gefriergerate-Kuhlschrankteile/_i.html?_sacat=184666"&gt;Gefriergeräte- &amp;amp; Kühlschrankteile&lt;/a&gt;
+                &lt;a class="footer-item" href="https://www.ebay.de/str/bremenhaushalt/Geschirrspulerteile/_i.html?_sacat=116026"&gt;Geschirrspülerteile&lt;/a&gt;
+                &lt;a class="footer-item" href="https://www.ebay.de/str/bremenhaushalt/Ersatzteile/_i.html?_sacat=99565"&gt;Kaffeemaschinen Ersatzteile&lt;/a&gt;
+                &lt;a class="footer-item" href="https://www.ebay.de/str/bremenhaushalt/Dunstabzugshauben/_i.html?_sacat=71253"&gt;Dunstabzugshauben Ersatzteile&lt;/a&gt;
+            &lt;/div&gt;
+        &lt;/div&gt;
+    &lt;/footer&gt;
+&lt;/div&gt;
+&lt;div class="container-fluid content-bg" align="center"&gt;
+    &lt;br/&gt;
+    &lt;div class="container"&gt;
+        &lt;div class="row"&gt;
+            &lt;div class="col-md-12 maincontent"&gt;
+                &lt;div class="row top_head"&gt;
+                    &lt;h1&gt;&lt;b style="color:#ff0000"&gt;Spannrolle wie Bosch 00600436 für Zweibandmotor Trockner&lt;/b&gt;&lt;/h1&gt;
+                &lt;/div&gt;
+                &lt;div class="textbox main"&gt;
+                    &lt;div class="row artdesc"&gt;
+                        &lt;div class="col-md-6 artdesc-2"&gt;
+                            &lt;div class="image-gallery"&gt;
+                                &lt;div class="big-image"&gt;
+                                    &lt;img id="default" src="https://4457.test1.ysell.pro/product_images/8/p-1-69678_1-1_info.jpg"/&gt;
+                                &lt;/div&gt;
+                            &lt;/div&gt;
+                        &lt;/div&gt;
+                        &lt;div class="col-md-6 artdesc-3"&gt;
+                            &lt;div class="right_info"&gt;
+                                &lt;div class="row"&gt;
+                                    &lt;div class="col"&gt;
+                                        &lt;a href="#" class="button-1" id="ersatz-tocart"&gt;
+                                            &lt;img src="https://ersatzteil-check.de/ebay_template/img/cart.svg" alt=""&gt;
+                                            Kaufen
+                                        &lt;/a&gt;
+                                    &lt;/div&gt;
+                                    &lt;div class="col"&gt;
+                                        &lt;a href="#" class="button-2" id="ersatz-towatch"&gt;
+                                            &lt;img src="https://ersatzteil-check.de/ebay_template/img/globalization.svg" alt=""&gt;
+                                            Beobachten
+                                        &lt;/a&gt;
+                                    &lt;/div&gt;
+                                    &lt;div class="col"&gt;
+                                        &lt;a href="#" class="button-3" id="ersatz-toask"&gt;
+                                            &lt;img src="https://ersatzteil-check.de/ebay_template/img/support.svg" alt=""&gt;
+                                            Frage stellen
+                                        &lt;/a&gt;
+                                    &lt;/div&gt;
+                                &lt;/div&gt;
+                                &lt;ul style="list-style-type:none; padding-left:0;"&gt;
+                                    &lt;li style="color:#ff0000;font-weight:700"&gt;&amp;#9989; &lt;b&gt;Originalgetreue Passform:&lt;/b&gt; Passend als Ersatz für Artikel-Nr.: 00600436&lt;/li&gt;
+                                    &lt;li style="color:#ff0000;font-weight:700"&gt;&amp;#9989; &lt;b&gt;Vielseitig einsetzbar:&lt;/b&gt; Kompatibel mit Produkten der Marke(n): Bosch&lt;/li&gt;
+                                    &lt;li style="color:#ff0000;font-weight:700"&gt;&amp;#9989; &lt;b&gt;Geprüfte Qualität:&lt;/b&gt; Hochwertige Verarbeitung in vergleichbarer Hersteller-Qualität&lt;/li&gt;
+                                    &lt;li style="color:#ff0000;font-weight:700"&gt;&amp;#9989; &lt;b&gt;Schnelle Lösung:&lt;/b&gt; Direkter Austausch ohne Modifikation möglich&lt;/li&gt;
+                                    &lt;li style="color:#ff0000;font-weight:700"&gt;&amp;#9989; &lt;b&gt;Sind Sie unsicher?&lt;/b&gt; Wir helfen Ihnen gerne, das exakt benötigte Ersatzteil zu finden.&lt;/li&gt;
+                                &lt;/ul&gt;
+                            &lt;/div&gt;
+                        &lt;/div&gt;
+                    &lt;/div&gt;
+                &lt;/div&gt;
+                &lt;div class="row bottom_text"&gt;
+                    &lt;div class="col-md-12"&gt;
+                        &lt;div class="tbc-1"&gt;
+                            &lt;h2&gt;Beschreibung&lt;/h2&gt;
+                            &lt;b style="color:#ff0000"&gt;Spannrolle wie Bosch 00600436 für Zweibandmotor Trockner&lt;/b&gt;&lt;br/&gt;&lt;br/&gt;
+                            &lt;span style="color:#ff0000"&gt;Dieser Artikel ist ein hochwertiges Ersatzteil, das kompatibel mit Geräten der Marke(n) Bosch ist. Er entspricht den Original-Spezifikationen und eignet sich als direkter Austausch.&lt;/span&gt;&lt;br/&gt;&lt;br/&gt;
+                            Wir sind ein professioneller Hersteller und Vertreiber von Original-Ersatzteilen und Alternativprodukten für Haushaltsgeräte. Egal ob Waschmaschine, Herd oder Kühlschrank: Wir haben diverse preisgünstige Original- und Alternativteile in vergleichbarer Hersteller-Qualität im Angebot. Überzeugen Sie sich selbst von der Wertigkeit unserer Ersatzteile und verschaffen Sie Ihrem Haushaltsgerät ein zweites Leben.&lt;br/&gt;&lt;br/&gt;
+                            &lt;b&gt;Kompatibel mit:&lt;/b&gt;&lt;br/&gt;
+                            &lt;span style="color:#ff0000"&gt;00600436&lt;/span&gt;
+                        &lt;/div&gt;
+                    &lt;/div&gt;
+                &lt;/div&gt;
+                &lt;div class="row bottom_text"&gt;
+                    &lt;div class="col-md-12"&gt;
+                        &lt;div class="tbc-2"&gt;
+                            &lt;h2&gt;Zahlungsoptionen&lt;/h2&gt;
+                            &lt;img src="https://ersatzteil-check.de/ebay_template/img/zahlung-paypal_n.png"&gt;
+                            &lt;img src="https://ersatzteil-check.de/ebay_template/img/zahlung-ueberweisung_n.png"&gt;
+                        &lt;/div&gt;
+                        &lt;div class="tbc-3"&gt;
+                            &lt;h2&gt;Versandoptionen&lt;/h2&gt;
+                            &lt;img src="https://ersatzteil-check.de/ebay_template/img/versand-dhl_n.png"&gt;
+                        &lt;/div&gt;
+                    &lt;/div&gt;
+                &lt;/div&gt;
+            &lt;/div&gt;
+        &lt;/div&gt;
+    &lt;/div&gt;
+&lt;/div&gt;
+&lt;/body&gt;
+&lt;/html&gt;</t>
+  </si>
+  <si>
     <t>Spannrolle wie Bosch 00600436 für Zweibandmotor Trockner</t>
   </si>
   <si>
@@ -179,6 +596,144 @@
     <t>p-4457-5</t>
   </si>
   <si>
+    <t>&lt;!DOCTYPE html&gt;
+&lt;html&gt;
+&lt;head&gt;
+    &lt;meta charset="utf-8"&gt;
+    &lt;meta name="viewport" content="width=device-width, initial-scale=1"&gt;
+    &lt;title&gt;eBay&lt;/title&gt;
+    &lt;link rel="preconnect" href="https://fonts.googleapis.com"&gt;
+    &lt;link rel="preconnect" href="https://fonts.gstatic.com" crossorigin&gt;
+    &lt;link href="https://fonts.googleapis.com/css2?family=Inter:wght@400;600&amp;display=swap" rel="stylesheet"&gt;
+    &lt;link rel="stylesheet" href="https://ersatzteil-check.de/ebay_template/css/style.css"&gt;
+    &lt;link rel="stylesheet" href="https://ersatzteil-check.de/ebay_template/css/new_style.css"&gt;
+    &lt;link href="https://cdn.jsdelivr.net/npm/bootstrap@5.3.2/dist/css/bootstrap.min.css" rel="stylesheet" crossorigin="anonymous"&gt;
+&lt;/head&gt;
+&lt;body&gt;
+&lt;div class="ebay-content"&gt;
+    &lt;header class="container header"&gt;
+        &lt;img src="https://ersatzteil-check.de/ebay_template/img/logo.svg"&gt;
+        &lt;div class="menu"&gt;
+            &lt;a class="menu-item" href="https://www.ebay.de/str/bremenhaushalt"&gt;Über uns&lt;/a&gt;
+            &lt;a class="menu-item" href="https://www.ebay.de/cnt/intermediatedFAQ?requested=ersatzteil-check-de"&gt;Kontakt&lt;/a&gt;
+            &lt;a class="menu-item" href="https://www.ebay.de/str/bremenhaushalt?_tab=2"&gt;Bewertungen&lt;/a&gt;
+            &lt;a class="menu-item-btn" href="https://www.ebay.de/str/bremenhaushalt"&gt;eBay Shop&lt;/a&gt;
+        &lt;/div&gt;
+    &lt;/header&gt;
+    &lt;div class="container"&gt;
+        &lt;img class="banner" src="https://ersatzteil-check.de/ebay_template/img/banner.png"&gt;
+    &lt;/div&gt;
+    &lt;div class="container gears"&gt;
+        &lt;div class="column-3"&gt;
+            &lt;img src="https://ersatzteil-check.de/ebay_template/img/Group1.png"&gt;
+            &lt;p&gt;Schnelle Lieferung&lt;/p&gt;
+        &lt;/div&gt;
+        &lt;div class="column-3"&gt;
+            &lt;img src="https://ersatzteil-check.de/ebay_template/img/Group2.png"&gt;
+            &lt;p&gt;Riesige Auswahl&lt;/p&gt;
+        &lt;/div&gt;
+        &lt;div class="column-3"&gt;
+            &lt;img src="https://ersatzteil-check.de/ebay_template/img/Group3.png"&gt;
+            &lt;p&gt;30 Tage Widerruffrist&lt;/p&gt;
+        &lt;/div&gt;
+    &lt;/div&gt;
+    &lt;footer class="footer"&gt;
+        &lt;div class="container"&gt;
+            &lt;div class="footer-menu"&gt;
+                &lt;a class="footer-item" href="https://www.ebay.de/sch/i.html?_ssn=ersatzteil-check-de&amp;store_name=bremenhaushalt&amp;_oac=1&amp;_trksid=p4429486.m3561.l2562"&gt;Alle Artikel&lt;/a&gt;
+                &lt;a class="footer-item" href="https://www.ebay.de/str/bremenhaushalt/Backofen-Herdteile/_i.html?_sacat=43566"&gt;Backofen- &amp;amp; Herdeteile&lt;/a&gt;
+                &lt;a class="footer-item" href="https://www.ebay.de/str/bremenhaushalt/Waschmaschinen-Trocknerteile/_i.html?_sacat=99697"&gt;Waschmaschinen- &amp;amp; Trocknerteile&lt;/a&gt;
+                &lt;a class="footer-item" href="https://www.ebay.de/str/bremenhaushalt/Gefriergerate-Kuhlschrankteile/_i.html?_sacat=184666"&gt;Gefriergeräte- &amp;amp; Kühlschrankteile&lt;/a&gt;
+                &lt;a class="footer-item" href="https://www.ebay.de/str/bremenhaushalt/Geschirrspulerteile/_i.html?_sacat=116026"&gt;Geschirrspülerteile&lt;/a&gt;
+                &lt;a class="footer-item" href="https://www.ebay.de/str/bremenhaushalt/Ersatzteile/_i.html?_sacat=99565"&gt;Kaffeemaschinen Ersatzteile&lt;/a&gt;
+                &lt;a class="footer-item" href="https://www.ebay.de/str/bremenhaushalt/Dunstabzugshauben/_i.html?_sacat=71253"&gt;Dunstabzugshauben Ersatzteile&lt;/a&gt;
+            &lt;/div&gt;
+        &lt;/div&gt;
+    &lt;/footer&gt;
+&lt;/div&gt;
+&lt;div class="container-fluid content-bg" align="center"&gt;
+    &lt;br/&gt;
+    &lt;div class="container"&gt;
+        &lt;div class="row"&gt;
+            &lt;div class="col-md-12 maincontent"&gt;
+                &lt;div class="row top_head"&gt;
+                    &lt;h1&gt;&lt;b style="color:#ff0000"&gt;Heizung Oberhitze SoftGrill wie IGNIS 488000525918 EGO 20.40943.000 Bauknecht 488000525918 481225998522 481225998472 für Herd Backofen&lt;/b&gt;&lt;/h1&gt;
+                &lt;/div&gt;
+                &lt;div class="textbox main"&gt;
+                    &lt;div class="row artdesc"&gt;
+                        &lt;div class="col-md-6 artdesc-2"&gt;
+                            &lt;div class="image-gallery"&gt;
+                                &lt;div class="big-image"&gt;
+                                    &lt;img id="default" src="https://4457.test1.ysell.pro/product_images/5/p-1-66796_1-2_info_DE.jpg"/&gt;
+                                &lt;/div&gt;
+                            &lt;/div&gt;
+                        &lt;/div&gt;
+                        &lt;div class="col-md-6 artdesc-3"&gt;
+                            &lt;div class="right_info"&gt;
+                                &lt;div class="row"&gt;
+                                    &lt;div class="col"&gt;
+                                        &lt;a href="#" class="button-1" id="ersatz-tocart"&gt;
+                                            &lt;img src="https://ersatzteil-check.de/ebay_template/img/cart.svg" alt=""&gt;
+                                            Kaufen
+                                        &lt;/a&gt;
+                                    &lt;/div&gt;
+                                    &lt;div class="col"&gt;
+                                        &lt;a href="#" class="button-2" id="ersatz-towatch"&gt;
+                                            &lt;img src="https://ersatzteil-check.de/ebay_template/img/globalization.svg" alt=""&gt;
+                                            Beobachten
+                                        &lt;/a&gt;
+                                    &lt;/div&gt;
+                                    &lt;div class="col"&gt;
+                                        &lt;a href="#" class="button-3" id="ersatz-toask"&gt;
+                                            &lt;img src="https://ersatzteil-check.de/ebay_template/img/support.svg" alt=""&gt;
+                                            Frage stellen
+                                        &lt;/a&gt;
+                                    &lt;/div&gt;
+                                &lt;/div&gt;
+                                &lt;ul style="list-style-type:none; padding-left:0;"&gt;
+                                    &lt;li style="color:#ff0000;font-weight:700"&gt;&amp;#9989; &lt;b&gt;Originalgetreue Passform:&lt;/b&gt; Passend als Ersatz für Artikel-Nr.: 488000525918, 20.40943.000, 481225998522&lt;/li&gt;
+                                    &lt;li style="color:#ff0000;font-weight:700"&gt;&amp;#9989; &lt;b&gt;Vielseitig einsetzbar:&lt;/b&gt; Kompatibel mit Produkten der Marke(n): IGNIS, EGO, Bauknecht&lt;/li&gt;
+                                    &lt;li style="color:#ff0000;font-weight:700"&gt;&amp;#9989; &lt;b&gt;Geprüfte Qualität:&lt;/b&gt; Hochwertige Verarbeitung in vergleichbarer Hersteller-Qualität&lt;/li&gt;
+                                    &lt;li style="color:#ff0000;font-weight:700"&gt;&amp;#9989; &lt;b&gt;Schnelle Lösung:&lt;/b&gt; Direkter Austausch ohne Modifikation möglich&lt;/li&gt;
+                                    &lt;li style="color:#ff0000;font-weight:700"&gt;&amp;#9989; &lt;b&gt;Sind Sie unsicher?&lt;/b&gt; Wir helfen Ihnen gerne, das exakt benötigte Ersatzteil zu finden.&lt;/li&gt;
+                                &lt;/ul&gt;
+                            &lt;/div&gt;
+                        &lt;/div&gt;
+                    &lt;/div&gt;
+                &lt;/div&gt;
+                &lt;div class="row bottom_text"&gt;
+                    &lt;div class="col-md-12"&gt;
+                        &lt;div class="tbc-1"&gt;
+                            &lt;h2&gt;Beschreibung&lt;/h2&gt;
+                            &lt;b style="color:#ff0000"&gt;Heizung Oberhitze SoftGrill wie IGNIS 488000525918 EGO 20.40943.000 Bauknecht 488000525918 481225998522 481225998472 für Herd Backofen&lt;/b&gt;&lt;br/&gt;&lt;br/&gt;
+                            &lt;span style="color:#ff0000"&gt;Dieser Artikel ist ein hochwertiges Ersatzteil, das kompatibel mit Geräten der Marke(n) IGNIS, EGO, Bauknecht ist. Er entspricht den Original-Spezifikationen und eignet sich als direkter Austausch.&lt;/span&gt;&lt;br/&gt;&lt;br/&gt;
+                            Wir sind ein professioneller Hersteller und Vertreiber von Original-Ersatzteilen und Alternativprodukten für Haushaltsgeräte. Egal ob Waschmaschine, Herd oder Kühlschrank: Wir haben diverse preisgünstige Original- und Alternativteile in vergleichbarer Hersteller-Qualität im Angebot. Überzeugen Sie sich selbst von der Wertigkeit unserer Ersatzteile und verschaffen Sie Ihrem Haushaltsgerät ein zweites Leben.&lt;br/&gt;&lt;br/&gt;
+                            &lt;b&gt;Kompatibel mit:&lt;/b&gt;&lt;br/&gt;
+                            &lt;span style="color:#ff0000"&gt;488000525918&lt;br/&gt;20.40943.000&lt;br/&gt;481225998522&lt;/span&gt;
+                        &lt;/div&gt;
+                    &lt;/div&gt;
+                &lt;/div&gt;
+                &lt;div class="row bottom_text"&gt;
+                    &lt;div class="col-md-12"&gt;
+                        &lt;div class="tbc-2"&gt;
+                            &lt;h2&gt;Zahlungsoptionen&lt;/h2&gt;
+                            &lt;img src="https://ersatzteil-check.de/ebay_template/img/zahlung-paypal_n.png"&gt;
+                            &lt;img src="https://ersatzteil-check.de/ebay_template/img/zahlung-ueberweisung_n.png"&gt;
+                        &lt;/div&gt;
+                        &lt;div class="tbc-3"&gt;
+                            &lt;h2&gt;Versandoptionen&lt;/h2&gt;
+                            &lt;img src="https://ersatzteil-check.de/ebay_template/img/versand-dhl_n.png"&gt;
+                        &lt;/div&gt;
+                    &lt;/div&gt;
+                &lt;/div&gt;
+            &lt;/div&gt;
+        &lt;/div&gt;
+    &lt;/div&gt;
+&lt;/div&gt;
+&lt;/body&gt;
+&lt;/html&gt;</t>
+  </si>
+  <si>
     <t>Heizung Oberhitze SoftGrill wie IGNIS 488000525918 EGO 20.40943.000 Bauknecht 48</t>
   </si>
   <si>
@@ -195,6 +750,144 @@
   </si>
   <si>
     <t>12-MP</t>
+  </si>
+  <si>
+    <t>&lt;!DOCTYPE html&gt;
+&lt;html&gt;
+&lt;head&gt;
+    &lt;meta charset="utf-8"&gt;
+    &lt;meta name="viewport" content="width=device-width, initial-scale=1"&gt;
+    &lt;title&gt;eBay&lt;/title&gt;
+    &lt;link rel="preconnect" href="https://fonts.googleapis.com"&gt;
+    &lt;link rel="preconnect" href="https://fonts.gstatic.com" crossorigin&gt;
+    &lt;link href="https://fonts.googleapis.com/css2?family=Inter:wght@400;600&amp;display=swap" rel="stylesheet"&gt;
+    &lt;link rel="stylesheet" href="https://ersatzteil-check.de/ebay_template/css/style.css"&gt;
+    &lt;link rel="stylesheet" href="https://ersatzteil-check.de/ebay_template/css/new_style.css"&gt;
+    &lt;link href="https://cdn.jsdelivr.net/npm/bootstrap@5.3.2/dist/css/bootstrap.min.css" rel="stylesheet" crossorigin="anonymous"&gt;
+&lt;/head&gt;
+&lt;body&gt;
+&lt;div class="ebay-content"&gt;
+    &lt;header class="container header"&gt;
+        &lt;img src="https://ersatzteil-check.de/ebay_template/img/logo.svg"&gt;
+        &lt;div class="menu"&gt;
+            &lt;a class="menu-item" href="https://www.ebay.de/str/bremenhaushalt"&gt;Über uns&lt;/a&gt;
+            &lt;a class="menu-item" href="https://www.ebay.de/cnt/intermediatedFAQ?requested=ersatzteil-check-de"&gt;Kontakt&lt;/a&gt;
+            &lt;a class="menu-item" href="https://www.ebay.de/str/bremenhaushalt?_tab=2"&gt;Bewertungen&lt;/a&gt;
+            &lt;a class="menu-item-btn" href="https://www.ebay.de/str/bremenhaushalt"&gt;eBay Shop&lt;/a&gt;
+        &lt;/div&gt;
+    &lt;/header&gt;
+    &lt;div class="container"&gt;
+        &lt;img class="banner" src="https://ersatzteil-check.de/ebay_template/img/banner.png"&gt;
+    &lt;/div&gt;
+    &lt;div class="container gears"&gt;
+        &lt;div class="column-3"&gt;
+            &lt;img src="https://ersatzteil-check.de/ebay_template/img/Group1.png"&gt;
+            &lt;p&gt;Schnelle Lieferung&lt;/p&gt;
+        &lt;/div&gt;
+        &lt;div class="column-3"&gt;
+            &lt;img src="https://ersatzteil-check.de/ebay_template/img/Group2.png"&gt;
+            &lt;p&gt;Riesige Auswahl&lt;/p&gt;
+        &lt;/div&gt;
+        &lt;div class="column-3"&gt;
+            &lt;img src="https://ersatzteil-check.de/ebay_template/img/Group3.png"&gt;
+            &lt;p&gt;30 Tage Widerruffrist&lt;/p&gt;
+        &lt;/div&gt;
+    &lt;/div&gt;
+    &lt;footer class="footer"&gt;
+        &lt;div class="container"&gt;
+            &lt;div class="footer-menu"&gt;
+                &lt;a class="footer-item" href="https://www.ebay.de/sch/i.html?_ssn=ersatzteil-check-de&amp;store_name=bremenhaushalt&amp;_oac=1&amp;_trksid=p4429486.m3561.l2562"&gt;Alle Artikel&lt;/a&gt;
+                &lt;a class="footer-item" href="https://www.ebay.de/str/bremenhaushalt/Backofen-Herdteile/_i.html?_sacat=43566"&gt;Backofen- &amp;amp; Herdeteile&lt;/a&gt;
+                &lt;a class="footer-item" href="https://www.ebay.de/str/bremenhaushalt/Waschmaschinen-Trocknerteile/_i.html?_sacat=99697"&gt;Waschmaschinen- &amp;amp; Trocknerteile&lt;/a&gt;
+                &lt;a class="footer-item" href="https://www.ebay.de/str/bremenhaushalt/Gefriergerate-Kuhlschrankteile/_i.html?_sacat=184666"&gt;Gefriergeräte- &amp;amp; Kühlschrankteile&lt;/a&gt;
+                &lt;a class="footer-item" href="https://www.ebay.de/str/bremenhaushalt/Geschirrspulerteile/_i.html?_sacat=116026"&gt;Geschirrspülerteile&lt;/a&gt;
+                &lt;a class="footer-item" href="https://www.ebay.de/str/bremenhaushalt/Ersatzteile/_i.html?_sacat=99565"&gt;Kaffeemaschinen Ersatzteile&lt;/a&gt;
+                &lt;a class="footer-item" href="https://www.ebay.de/str/bremenhaushalt/Dunstabzugshauben/_i.html?_sacat=71253"&gt;Dunstabzugshauben Ersatzteile&lt;/a&gt;
+            &lt;/div&gt;
+        &lt;/div&gt;
+    &lt;/footer&gt;
+&lt;/div&gt;
+&lt;div class="container-fluid content-bg" align="center"&gt;
+    &lt;br/&gt;
+    &lt;div class="container"&gt;
+        &lt;div class="row"&gt;
+            &lt;div class="col-md-12 maincontent"&gt;
+                &lt;div class="row top_head"&gt;
+                    &lt;h1&gt;&lt;b style="color:#ff0000"&gt;Bosch Siemens 17002715 / 17001433 Backblech Fettpfanne Grillpfanne 455x375x39(33)mm für Herd&lt;/b&gt;&lt;/h1&gt;
+                &lt;/div&gt;
+                &lt;div class="textbox main"&gt;
+                    &lt;div class="row artdesc"&gt;
+                        &lt;div class="col-md-6 artdesc-2"&gt;
+                            &lt;div class="image-gallery"&gt;
+                                &lt;div class="big-image"&gt;
+                                    &lt;img id="default" src="https://4457.test1.ysell.pro/product_images/12/13682.jpg"/&gt;
+                                &lt;/div&gt;
+                            &lt;/div&gt;
+                        &lt;/div&gt;
+                        &lt;div class="col-md-6 artdesc-3"&gt;
+                            &lt;div class="right_info"&gt;
+                                &lt;div class="row"&gt;
+                                    &lt;div class="col"&gt;
+                                        &lt;a href="#" class="button-1" id="ersatz-tocart"&gt;
+                                            &lt;img src="https://ersatzteil-check.de/ebay_template/img/cart.svg" alt=""&gt;
+                                            Kaufen
+                                        &lt;/a&gt;
+                                    &lt;/div&gt;
+                                    &lt;div class="col"&gt;
+                                        &lt;a href="#" class="button-2" id="ersatz-towatch"&gt;
+                                            &lt;img src="https://ersatzteil-check.de/ebay_template/img/globalization.svg" alt=""&gt;
+                                            Beobachten
+                                        &lt;/a&gt;
+                                    &lt;/div&gt;
+                                    &lt;div class="col"&gt;
+                                        &lt;a href="#" class="button-3" id="ersatz-toask"&gt;
+                                            &lt;img src="https://ersatzteil-check.de/ebay_template/img/support.svg" alt=""&gt;
+                                            Frage stellen
+                                        &lt;/a&gt;
+                                    &lt;/div&gt;
+                                &lt;/div&gt;
+                                &lt;ul style="list-style-type:none; padding-left:0;"&gt;
+                                    &lt;li style="color:#ff0000;font-weight:700"&gt;&amp;#9989; &lt;b&gt;Originalgetreue Passform:&lt;/b&gt; Passend als Ersatz für Artikel-Nr.: 17002715, 17001433&lt;/li&gt;
+                                    &lt;li style="color:#ff0000;font-weight:700"&gt;&amp;#9989; &lt;b&gt;Vielseitig einsetzbar:&lt;/b&gt; Geeignet als Ersatzteil für viele gängige Haushaltsgeräte&lt;/li&gt;
+                                    &lt;li style="color:#ff0000;font-weight:700"&gt;&amp;#9989; &lt;b&gt;Geprüfte Qualität:&lt;/b&gt; Hochwertige Verarbeitung in vergleichbarer Hersteller-Qualität&lt;/li&gt;
+                                    &lt;li style="color:#ff0000;font-weight:700"&gt;&amp;#9989; &lt;b&gt;Schnelle Lösung:&lt;/b&gt; Direkter Austausch ohne Modifikation möglich&lt;/li&gt;
+                                    &lt;li style="color:#ff0000;font-weight:700"&gt;&amp;#9989; &lt;b&gt;Sind Sie unsicher?&lt;/b&gt; Wir helfen Ihnen gerne, das exakt benötigte Ersatzteil zu finden.&lt;/li&gt;
+                                &lt;/ul&gt;
+                            &lt;/div&gt;
+                        &lt;/div&gt;
+                    &lt;/div&gt;
+                &lt;/div&gt;
+                &lt;div class="row bottom_text"&gt;
+                    &lt;div class="col-md-12"&gt;
+                        &lt;div class="tbc-1"&gt;
+                            &lt;h2&gt;Beschreibung&lt;/h2&gt;
+                            &lt;b style="color:#ff0000"&gt;Bosch Siemens 17002715 / 17001433 Backblech Fettpfanne Grillpfanne 455x375x39(33)mm für Herd&lt;/b&gt;&lt;br/&gt;&lt;br/&gt;
+                            &lt;span style="color:#ff0000"&gt;Dieser Artikel ist ein hochwertiges Ersatzteil für Haushaltsgeräte. Er entspricht den Original-Spezifikationen und eignet sich als direkter Austausch.&lt;/span&gt;&lt;br/&gt;&lt;br/&gt;
+                            Wir sind ein professioneller Hersteller und Vertreiber von Original-Ersatzteilen und Alternativprodukten für Haushaltsgeräte. Egal ob Waschmaschine, Herd oder Kühlschrank: Wir haben diverse preisgünstige Original- und Alternativteile in vergleichbarer Hersteller-Qualität im Angebot. Überzeugen Sie sich selbst von der Wertigkeit unserer Ersatzteile und verschaffen Sie Ihrem Haushaltsgerät ein zweites Leben.&lt;br/&gt;&lt;br/&gt;
+                            &lt;b&gt;Kompatibel mit:&lt;/b&gt;&lt;br/&gt;
+                            &lt;span style="color:#ff0000"&gt;17002715&lt;br/&gt;17001433&lt;/span&gt;
+                        &lt;/div&gt;
+                    &lt;/div&gt;
+                &lt;/div&gt;
+                &lt;div class="row bottom_text"&gt;
+                    &lt;div class="col-md-12"&gt;
+                        &lt;div class="tbc-2"&gt;
+                            &lt;h2&gt;Zahlungsoptionen&lt;/h2&gt;
+                            &lt;img src="https://ersatzteil-check.de/ebay_template/img/zahlung-paypal_n.png"&gt;
+                            &lt;img src="https://ersatzteil-check.de/ebay_template/img/zahlung-ueberweisung_n.png"&gt;
+                        &lt;/div&gt;
+                        &lt;div class="tbc-3"&gt;
+                            &lt;h2&gt;Versandoptionen&lt;/h2&gt;
+                            &lt;img src="https://ersatzteil-check.de/ebay_template/img/versand-dhl_n.png"&gt;
+                        &lt;/div&gt;
+                    &lt;/div&gt;
+                &lt;/div&gt;
+            &lt;/div&gt;
+        &lt;/div&gt;
+    &lt;/div&gt;
+&lt;/div&gt;
+&lt;/body&gt;
+&lt;/html&gt;</t>
   </si>
   <si>
     <t>Bosch Siemens 17002715 / 17001433 Backblech Fettpfanne Grillpfanne 455x375x39(33</t>
@@ -553,37 +1246,38 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:Y6"/>
+  <dimension ref="A1:Z6"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="9.283" customWidth="true" style="0"/>
     <col min="2" max="2" width="22.28" customWidth="true" style="0"/>
     <col min="3" max="3" width="11.711" customWidth="true" style="0"/>
-    <col min="4" max="4" width="8.141" customWidth="true" style="0"/>
-    <col min="5" max="5" width="15.282" customWidth="true" style="0"/>
-    <col min="6" max="6" width="24.708" customWidth="true" style="0"/>
-    <col min="7" max="7" width="13.997" customWidth="true" style="0"/>
-    <col min="8" max="8" width="11.711" customWidth="true" style="0"/>
-    <col min="9" max="9" width="9.283" customWidth="true" style="0"/>
-    <col min="10" max="10" width="11.711" customWidth="true" style="0"/>
+    <col min="4" max="4" width="13.997" customWidth="true" style="0"/>
+    <col min="5" max="5" width="8.141" customWidth="true" style="0"/>
+    <col min="6" max="6" width="15.282" customWidth="true" style="0"/>
+    <col min="7" max="7" width="24.708" customWidth="true" style="0"/>
+    <col min="8" max="8" width="13.997" customWidth="true" style="0"/>
+    <col min="9" max="9" width="11.711" customWidth="true" style="0"/>
+    <col min="10" max="10" width="9.283" customWidth="true" style="0"/>
     <col min="11" max="11" width="11.711" customWidth="true" style="0"/>
-    <col min="12" max="12" width="23.423" customWidth="true" style="0"/>
-    <col min="13" max="13" width="21.138" customWidth="true" style="0"/>
-    <col min="14" max="14" width="22.28" customWidth="true" style="0"/>
-    <col min="15" max="15" width="8.141" customWidth="true" style="0"/>
-    <col min="16" max="16" width="9.283" customWidth="true" style="0"/>
-    <col min="17" max="17" width="15.282" customWidth="true" style="0"/>
+    <col min="12" max="12" width="11.711" customWidth="true" style="0"/>
+    <col min="13" max="13" width="23.423" customWidth="true" style="0"/>
+    <col min="14" max="14" width="21.138" customWidth="true" style="0"/>
+    <col min="15" max="15" width="22.28" customWidth="true" style="0"/>
+    <col min="16" max="16" width="8.141" customWidth="true" style="0"/>
+    <col min="17" max="17" width="9.283" customWidth="true" style="0"/>
     <col min="18" max="18" width="15.282" customWidth="true" style="0"/>
-    <col min="19" max="19" width="11.711" customWidth="true" style="0"/>
-    <col min="20" max="20" width="9.283" customWidth="true" style="0"/>
-    <col min="21" max="21" width="12.854" customWidth="true" style="0"/>
-    <col min="22" max="22" width="26.993" customWidth="true" style="0"/>
+    <col min="19" max="19" width="15.282" customWidth="true" style="0"/>
+    <col min="20" max="20" width="11.711" customWidth="true" style="0"/>
+    <col min="21" max="21" width="9.283" customWidth="true" style="0"/>
+    <col min="22" max="22" width="12.854" customWidth="true" style="0"/>
     <col min="23" max="23" width="26.993" customWidth="true" style="0"/>
-    <col min="24" max="24" width="22.28" customWidth="true" style="0"/>
+    <col min="24" max="24" width="26.993" customWidth="true" style="0"/>
     <col min="25" max="25" width="22.28" customWidth="true" style="0"/>
+    <col min="26" max="26" width="22.28" customWidth="true" style="0"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:25">
+    <row r="1" spans="1:26">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -659,333 +1353,366 @@
       <c r="Y1" s="1" t="s">
         <v>24</v>
       </c>
+      <c r="Z1" t="s">
+        <v>25</v>
+      </c>
     </row>
-    <row r="2" spans="1:25">
+    <row r="2" spans="1:26">
       <c r="A2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C2">
+        <v>99565</v>
+      </c>
+      <c r="D2" t="s">
+        <v>28</v>
+      </c>
+      <c r="E2" t="s">
+        <v>29</v>
+      </c>
+      <c r="F2">
+        <v>1000</v>
+      </c>
+      <c r="G2" t="s">
+        <v>30</v>
+      </c>
+      <c r="I2">
+        <v>1</v>
+      </c>
+      <c r="J2" t="s">
+        <v>31</v>
+      </c>
+      <c r="K2" t="s">
+        <v>32</v>
+      </c>
+      <c r="L2" t="s">
+        <v>33</v>
+      </c>
+      <c r="M2" t="s">
+        <v>34</v>
+      </c>
+      <c r="N2" t="s">
+        <v>35</v>
+      </c>
+      <c r="O2" t="s">
+        <v>36</v>
+      </c>
+      <c r="P2" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>38</v>
+      </c>
+      <c r="R2" t="s">
+        <v>38</v>
+      </c>
+      <c r="S2" t="s">
+        <v>39</v>
+      </c>
+      <c r="T2" t="s">
+        <v>39</v>
+      </c>
+      <c r="X2" t="s">
+        <v>40</v>
+      </c>
+      <c r="Y2" t="s">
+        <v>40</v>
+      </c>
+      <c r="Z2" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="3" spans="1:26">
+      <c r="A3" t="s">
         <v>26</v>
       </c>
-      <c r="D2" t="s">
-        <v>27</v>
-      </c>
-      <c r="E2">
+      <c r="B3" t="s">
+        <v>42</v>
+      </c>
+      <c r="C3">
+        <v>184666</v>
+      </c>
+      <c r="D3" t="s">
+        <v>43</v>
+      </c>
+      <c r="E3" t="s">
+        <v>44</v>
+      </c>
+      <c r="F3">
         <v>1000</v>
       </c>
-      <c r="F2" t="s">
-        <v>28</v>
-      </c>
-      <c r="H2">
+      <c r="G3" t="s">
+        <v>30</v>
+      </c>
+      <c r="H3">
+        <v>3.74</v>
+      </c>
+      <c r="I3">
         <v>1</v>
       </c>
-      <c r="I2" t="s">
-        <v>29</v>
-      </c>
-      <c r="J2" t="s">
+      <c r="J3" t="s">
+        <v>31</v>
+      </c>
+      <c r="K3" t="s">
+        <v>32</v>
+      </c>
+      <c r="L3" t="s">
+        <v>33</v>
+      </c>
+      <c r="M3" t="s">
+        <v>34</v>
+      </c>
+      <c r="N3" t="s">
+        <v>35</v>
+      </c>
+      <c r="O3" t="s">
+        <v>36</v>
+      </c>
+      <c r="P3" t="s">
+        <v>45</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>46</v>
+      </c>
+      <c r="R3" t="s">
+        <v>46</v>
+      </c>
+      <c r="S3" t="s">
+        <v>47</v>
+      </c>
+      <c r="T3" t="s">
+        <v>47</v>
+      </c>
+      <c r="W3" t="s">
+        <v>48</v>
+      </c>
+      <c r="X3" t="s">
+        <v>49</v>
+      </c>
+      <c r="Y3">
+        <v>7433698</v>
+      </c>
+      <c r="Z3" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="4" spans="1:26">
+      <c r="A4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B4" t="s">
+        <v>50</v>
+      </c>
+      <c r="C4">
+        <v>99697</v>
+      </c>
+      <c r="D4" t="s">
+        <v>51</v>
+      </c>
+      <c r="E4" t="s">
+        <v>52</v>
+      </c>
+      <c r="F4">
+        <v>1000</v>
+      </c>
+      <c r="G4" t="s">
         <v>30</v>
       </c>
-      <c r="K2" t="s">
+      <c r="H4">
+        <v>3.96</v>
+      </c>
+      <c r="I4">
+        <v>1</v>
+      </c>
+      <c r="J4" t="s">
         <v>31</v>
       </c>
-      <c r="L2" t="s">
+      <c r="K4" t="s">
         <v>32</v>
       </c>
-      <c r="M2" t="s">
+      <c r="L4" t="s">
         <v>33</v>
       </c>
-      <c r="N2" t="s">
+      <c r="M4" t="s">
         <v>34</v>
       </c>
-      <c r="O2" t="s">
+      <c r="N4" t="s">
         <v>35</v>
       </c>
-      <c r="P2" t="s">
+      <c r="O4" t="s">
         <v>36</v>
       </c>
-      <c r="Q2" t="s">
+      <c r="P4" t="s">
+        <v>53</v>
+      </c>
+      <c r="Q4" t="s">
+        <v>46</v>
+      </c>
+      <c r="R4" t="s">
+        <v>46</v>
+      </c>
+      <c r="S4" t="s">
+        <v>54</v>
+      </c>
+      <c r="T4" t="s">
+        <v>54</v>
+      </c>
+      <c r="W4" t="s">
+        <v>55</v>
+      </c>
+      <c r="X4" t="s">
+        <v>56</v>
+      </c>
+      <c r="Y4" t="s">
+        <v>56</v>
+      </c>
+      <c r="Z4" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="5" spans="1:26">
+      <c r="A5" t="s">
+        <v>26</v>
+      </c>
+      <c r="B5" t="s">
+        <v>57</v>
+      </c>
+      <c r="C5">
+        <v>43566</v>
+      </c>
+      <c r="D5" t="s">
+        <v>58</v>
+      </c>
+      <c r="E5" t="s">
+        <v>59</v>
+      </c>
+      <c r="F5">
+        <v>1000</v>
+      </c>
+      <c r="G5" t="s">
+        <v>30</v>
+      </c>
+      <c r="I5">
+        <v>1</v>
+      </c>
+      <c r="J5" t="s">
+        <v>31</v>
+      </c>
+      <c r="K5" t="s">
+        <v>32</v>
+      </c>
+      <c r="L5" t="s">
+        <v>33</v>
+      </c>
+      <c r="M5" t="s">
+        <v>34</v>
+      </c>
+      <c r="N5" t="s">
+        <v>35</v>
+      </c>
+      <c r="O5" t="s">
         <v>36</v>
       </c>
-      <c r="R2" t="s">
-        <v>37</v>
-      </c>
-      <c r="S2" t="s">
-        <v>37</v>
-      </c>
-      <c r="W2" t="s">
+      <c r="P5" t="s">
+        <v>60</v>
+      </c>
+      <c r="Q5" t="s">
+        <v>46</v>
+      </c>
+      <c r="R5" t="s">
+        <v>46</v>
+      </c>
+      <c r="S5" t="s">
+        <v>61</v>
+      </c>
+      <c r="T5" t="s">
+        <v>61</v>
+      </c>
+      <c r="W5" t="s">
+        <v>62</v>
+      </c>
+      <c r="X5" t="s">
+        <v>63</v>
+      </c>
+      <c r="Y5">
+        <v>488000525918</v>
+      </c>
+      <c r="Z5" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="6" spans="1:26">
+      <c r="A6" t="s">
+        <v>26</v>
+      </c>
+      <c r="B6" t="s">
+        <v>64</v>
+      </c>
+      <c r="C6">
+        <v>43566</v>
+      </c>
+      <c r="D6" t="s">
+        <v>65</v>
+      </c>
+      <c r="E6" t="s">
+        <v>66</v>
+      </c>
+      <c r="F6">
+        <v>1000</v>
+      </c>
+      <c r="G6" t="s">
+        <v>30</v>
+      </c>
+      <c r="H6">
+        <v>18.19</v>
+      </c>
+      <c r="I6">
+        <v>1</v>
+      </c>
+      <c r="J6" t="s">
+        <v>31</v>
+      </c>
+      <c r="K6" t="s">
+        <v>32</v>
+      </c>
+      <c r="L6" t="s">
+        <v>33</v>
+      </c>
+      <c r="M6" t="s">
+        <v>34</v>
+      </c>
+      <c r="N6" t="s">
+        <v>35</v>
+      </c>
+      <c r="O6" t="s">
+        <v>36</v>
+      </c>
+      <c r="P6" t="s">
+        <v>67</v>
+      </c>
+      <c r="Q6" t="s">
         <v>38</v>
       </c>
-      <c r="X2" t="s">
+      <c r="R6" t="s">
         <v>38</v>
       </c>
-      <c r="Y2" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="3" spans="1:25">
-      <c r="A3" t="s">
-        <v>25</v>
-      </c>
-      <c r="B3" t="s">
-        <v>40</v>
-      </c>
-      <c r="D3" t="s">
+      <c r="S6" t="s">
+        <v>55</v>
+      </c>
+      <c r="T6" t="s">
+        <v>55</v>
+      </c>
+      <c r="X6" t="s">
+        <v>68</v>
+      </c>
+      <c r="Y6">
+        <v>17002715</v>
+      </c>
+      <c r="Z6" t="s">
         <v>41</v>
-      </c>
-      <c r="E3">
-        <v>1000</v>
-      </c>
-      <c r="F3" t="s">
-        <v>28</v>
-      </c>
-      <c r="G3">
-        <v>3.74</v>
-      </c>
-      <c r="H3">
-        <v>1</v>
-      </c>
-      <c r="I3" t="s">
-        <v>29</v>
-      </c>
-      <c r="J3" t="s">
-        <v>30</v>
-      </c>
-      <c r="K3" t="s">
-        <v>31</v>
-      </c>
-      <c r="L3" t="s">
-        <v>32</v>
-      </c>
-      <c r="M3" t="s">
-        <v>33</v>
-      </c>
-      <c r="N3" t="s">
-        <v>34</v>
-      </c>
-      <c r="O3" t="s">
-        <v>42</v>
-      </c>
-      <c r="P3" t="s">
-        <v>43</v>
-      </c>
-      <c r="Q3" t="s">
-        <v>43</v>
-      </c>
-      <c r="R3" t="s">
-        <v>44</v>
-      </c>
-      <c r="S3" t="s">
-        <v>44</v>
-      </c>
-      <c r="V3" t="s">
-        <v>45</v>
-      </c>
-      <c r="W3" t="s">
-        <v>46</v>
-      </c>
-      <c r="X3">
-        <v>7433698</v>
-      </c>
-      <c r="Y3" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="4" spans="1:25">
-      <c r="A4" t="s">
-        <v>25</v>
-      </c>
-      <c r="B4" t="s">
-        <v>47</v>
-      </c>
-      <c r="D4" t="s">
-        <v>48</v>
-      </c>
-      <c r="E4">
-        <v>1000</v>
-      </c>
-      <c r="F4" t="s">
-        <v>28</v>
-      </c>
-      <c r="G4">
-        <v>3.96</v>
-      </c>
-      <c r="H4">
-        <v>1</v>
-      </c>
-      <c r="I4" t="s">
-        <v>29</v>
-      </c>
-      <c r="J4" t="s">
-        <v>30</v>
-      </c>
-      <c r="K4" t="s">
-        <v>31</v>
-      </c>
-      <c r="L4" t="s">
-        <v>32</v>
-      </c>
-      <c r="M4" t="s">
-        <v>33</v>
-      </c>
-      <c r="N4" t="s">
-        <v>34</v>
-      </c>
-      <c r="O4" t="s">
-        <v>49</v>
-      </c>
-      <c r="P4" t="s">
-        <v>43</v>
-      </c>
-      <c r="Q4" t="s">
-        <v>43</v>
-      </c>
-      <c r="R4" t="s">
-        <v>50</v>
-      </c>
-      <c r="S4" t="s">
-        <v>50</v>
-      </c>
-      <c r="V4" t="s">
-        <v>51</v>
-      </c>
-      <c r="W4" t="s">
-        <v>52</v>
-      </c>
-      <c r="X4" t="s">
-        <v>52</v>
-      </c>
-      <c r="Y4" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="5" spans="1:25">
-      <c r="A5" t="s">
-        <v>25</v>
-      </c>
-      <c r="B5" t="s">
-        <v>53</v>
-      </c>
-      <c r="D5" t="s">
-        <v>54</v>
-      </c>
-      <c r="E5">
-        <v>1000</v>
-      </c>
-      <c r="F5" t="s">
-        <v>28</v>
-      </c>
-      <c r="H5">
-        <v>1</v>
-      </c>
-      <c r="I5" t="s">
-        <v>29</v>
-      </c>
-      <c r="J5" t="s">
-        <v>30</v>
-      </c>
-      <c r="K5" t="s">
-        <v>31</v>
-      </c>
-      <c r="L5" t="s">
-        <v>32</v>
-      </c>
-      <c r="M5" t="s">
-        <v>33</v>
-      </c>
-      <c r="N5" t="s">
-        <v>34</v>
-      </c>
-      <c r="O5" t="s">
-        <v>55</v>
-      </c>
-      <c r="P5" t="s">
-        <v>43</v>
-      </c>
-      <c r="Q5" t="s">
-        <v>43</v>
-      </c>
-      <c r="R5" t="s">
-        <v>56</v>
-      </c>
-      <c r="S5" t="s">
-        <v>56</v>
-      </c>
-      <c r="V5" t="s">
-        <v>57</v>
-      </c>
-      <c r="W5" t="s">
-        <v>58</v>
-      </c>
-      <c r="X5">
-        <v>488000525918</v>
-      </c>
-      <c r="Y5" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="6" spans="1:25">
-      <c r="A6" t="s">
-        <v>25</v>
-      </c>
-      <c r="B6" t="s">
-        <v>59</v>
-      </c>
-      <c r="D6" t="s">
-        <v>60</v>
-      </c>
-      <c r="E6">
-        <v>1000</v>
-      </c>
-      <c r="F6" t="s">
-        <v>28</v>
-      </c>
-      <c r="G6">
-        <v>18.19</v>
-      </c>
-      <c r="H6">
-        <v>1</v>
-      </c>
-      <c r="I6" t="s">
-        <v>29</v>
-      </c>
-      <c r="J6" t="s">
-        <v>30</v>
-      </c>
-      <c r="K6" t="s">
-        <v>31</v>
-      </c>
-      <c r="L6" t="s">
-        <v>32</v>
-      </c>
-      <c r="M6" t="s">
-        <v>33</v>
-      </c>
-      <c r="N6" t="s">
-        <v>34</v>
-      </c>
-      <c r="O6" t="s">
-        <v>61</v>
-      </c>
-      <c r="P6" t="s">
-        <v>36</v>
-      </c>
-      <c r="Q6" t="s">
-        <v>36</v>
-      </c>
-      <c r="R6" t="s">
-        <v>51</v>
-      </c>
-      <c r="S6" t="s">
-        <v>51</v>
-      </c>
-      <c r="W6" t="s">
-        <v>62</v>
-      </c>
-      <c r="X6">
-        <v>17002715</v>
-      </c>
-      <c r="Y6" t="s">
-        <v>39</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update generated output files (flat_filled.xlsx, products_raw.json)
Regenerated after adding productSuppliers to sample data.

https://claude.ai/code/session_013CC3uQiZgCtv7kaNkq2QqP
</commit_message>
<xml_diff>
--- a/flat_filled.xlsx
+++ b/flat_filled.xlsx
@@ -1447,9 +1447,6 @@
       <c r="G3" t="s">
         <v>30</v>
       </c>
-      <c r="H3">
-        <v>3.74</v>
-      </c>
       <c r="I3">
         <v>1</v>
       </c>
@@ -1520,9 +1517,6 @@
       </c>
       <c r="G4" t="s">
         <v>30</v>
-      </c>
-      <c r="H4">
-        <v>3.96</v>
       </c>
       <c r="I4">
         <v>1</v>

</xml_diff>